<commit_message>
pos mod by A.T.
pos modifieied by A.T.
</commit_message>
<xml_diff>
--- a/Bon_commande_Farnell.xlsx
+++ b/Bon_commande_Farnell.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/C820B532B41E2663/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antotauv\Documents\Projet_1A_2026\ENSEA_S6_PROJET_OSCILLO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0AA1431-846B-4561-AA81-660C6BC0BAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19658B6-743B-4BAB-812B-CEA4246EB59B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10890" xr2:uid="{830003BB-F479-4779-B7E8-97ECCAD99C8E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{830003BB-F479-4779-B7E8-97ECCAD99C8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -123,7 +123,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,16 +225,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -581,15 +578,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{227F4AA7-155C-4488-B19E-C729B3F465C8}">
   <dimension ref="A1:N12"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="13.5" customHeight="1">
+    <row r="1" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.600000000000001" customHeight="1"/>
-    <row r="3" spans="1:14" ht="17.45" customHeight="1">
+    <row r="2" spans="1:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:14" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -605,10 +605,10 @@
       <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
@@ -631,7 +631,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="42">
+    <row r="4" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>10</v>
       </c>
@@ -641,10 +641,10 @@
       <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>10</v>
       </c>
-      <c r="G4" s="6"/>
+      <c r="G4" s="5"/>
       <c r="H4" t="s">
         <v>16</v>
       </c>
@@ -664,7 +664,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="21">
+    <row r="5" spans="1:14" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>20</v>
       </c>
@@ -674,10 +674,10 @@
       <c r="E5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>5</v>
       </c>
-      <c r="G5" s="4"/>
+      <c r="G5" s="3"/>
       <c r="H5" t="s">
         <v>16</v>
       </c>
@@ -697,7 +697,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="41.45" customHeight="1">
+    <row r="6" spans="1:14" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>30</v>
       </c>
@@ -707,10 +707,10 @@
       <c r="E6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>1</v>
       </c>
-      <c r="G6" s="4"/>
+      <c r="G6" s="3"/>
       <c r="H6" t="s">
         <v>16</v>
       </c>
@@ -730,7 +730,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="38.450000000000003" customHeight="1">
+    <row r="7" spans="1:14" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>40</v>
       </c>
@@ -740,10 +740,10 @@
       <c r="E7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <v>5</v>
       </c>
-      <c r="G7" s="4"/>
+      <c r="G7" s="3"/>
       <c r="H7" t="s">
         <v>16</v>
       </c>
@@ -763,7 +763,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="21">
+    <row r="8" spans="1:14" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A8">
         <f>SUM(A7,10)</f>
         <v>50</v>
@@ -771,13 +771,13 @@
       <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <v>5</v>
       </c>
-      <c r="G8" s="4"/>
+      <c r="G8" s="3"/>
       <c r="H8" t="s">
         <v>16</v>
       </c>
@@ -797,7 +797,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="31.5">
+    <row r="9" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A9">
         <f>SUM(A8,10)</f>
         <v>60</v>
@@ -808,10 +808,10 @@
       <c r="E9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>5</v>
       </c>
-      <c r="G9" s="4"/>
+      <c r="G9" s="3"/>
       <c r="H9" t="s">
         <v>16</v>
       </c>
@@ -831,7 +831,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="53.1" customHeight="1">
+    <row r="10" spans="1:14" ht="53.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" ref="A10:A11" si="0">SUM(A9,10)</f>
         <v>70</v>
@@ -842,10 +842,10 @@
       <c r="E10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>1</v>
       </c>
-      <c r="G10" s="4"/>
+      <c r="G10" s="3"/>
       <c r="H10" t="s">
         <v>16</v>
       </c>
@@ -865,7 +865,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="42">
+    <row r="11" spans="1:14" ht="45" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>80</v>
@@ -876,10 +876,10 @@
       <c r="E11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>1</v>
       </c>
-      <c r="G11" s="4"/>
+      <c r="G11" s="3"/>
       <c r="H11" t="s">
         <v>16</v>
       </c>
@@ -899,10 +899,10 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E12" s="1"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
Nettoyage / suppresion fichiers inutiles
</commit_message>
<xml_diff>
--- a/Bon_commande_Farnell.xlsx
+++ b/Bon_commande_Farnell.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antotauv\Documents\Projet_1A_2026\ENSEA_S6_PROJET_OSCILLO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gokay\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19658B6-743B-4BAB-812B-CEA4246EB59B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{747659A8-F3DC-4BC0-BA71-29CB5F7C248D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{830003BB-F479-4779-B7E8-97ECCAD99C8E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{830003BB-F479-4779-B7E8-97ECCAD99C8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -123,7 +123,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,7 +173,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -220,6 +220,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -236,11 +249,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -577,19 +590,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{227F4AA7-155C-4488-B19E-C729B3F465C8}">
-  <dimension ref="A1:N12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="13.5" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:14" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="20.5" customHeight="1"/>
+    <row r="3" spans="1:13" ht="17.5" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -605,33 +618,32 @@
       <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="G3" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="H3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="N3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="21">
       <c r="A4">
         <v>10</v>
       </c>
@@ -641,30 +653,29 @@
       <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>10</v>
       </c>
-      <c r="G4" s="5"/>
+      <c r="G4" t="s">
+        <v>16</v>
+      </c>
       <c r="H4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" t="s">
         <v>17</v>
       </c>
-      <c r="J4">
+      <c r="I4">
         <v>0.5</v>
       </c>
+      <c r="J4" t="s">
+        <v>18</v>
+      </c>
       <c r="K4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L4" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="20.5" customHeight="1">
       <c r="A5">
         <v>20</v>
       </c>
@@ -677,27 +688,26 @@
       <c r="F5" s="3">
         <v>5</v>
       </c>
-      <c r="G5" s="3"/>
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
       <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s">
         <v>17</v>
       </c>
-      <c r="J5">
+      <c r="I5">
         <v>0.14899999999999999</v>
       </c>
+      <c r="J5" t="s">
+        <v>18</v>
+      </c>
       <c r="K5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="17.5" customHeight="1">
       <c r="A6">
         <v>30</v>
       </c>
@@ -710,27 +720,26 @@
       <c r="F6" s="3">
         <v>1</v>
       </c>
-      <c r="G6" s="3"/>
+      <c r="G6" t="s">
+        <v>16</v>
+      </c>
       <c r="H6" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" t="s">
         <v>17</v>
       </c>
-      <c r="J6">
+      <c r="I6">
         <v>0.79</v>
       </c>
+      <c r="J6" t="s">
+        <v>18</v>
+      </c>
       <c r="K6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="22.5" customHeight="1">
       <c r="A7">
         <v>40</v>
       </c>
@@ -743,27 +752,26 @@
       <c r="F7" s="3">
         <v>5</v>
       </c>
-      <c r="G7" s="3"/>
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
       <c r="H7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s">
         <v>17</v>
       </c>
-      <c r="J7">
+      <c r="I7">
         <v>0.218</v>
       </c>
+      <c r="J7" t="s">
+        <v>18</v>
+      </c>
       <c r="K7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L7" t="s">
-        <v>16</v>
-      </c>
-      <c r="M7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13">
       <c r="A8">
         <f>SUM(A7,10)</f>
         <v>50</v>
@@ -777,27 +785,26 @@
       <c r="F8" s="3">
         <v>5</v>
       </c>
-      <c r="G8" s="3"/>
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
       <c r="H8" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" t="s">
         <v>17</v>
       </c>
-      <c r="J8">
+      <c r="I8">
         <v>0.1</v>
       </c>
+      <c r="J8" t="s">
+        <v>18</v>
+      </c>
       <c r="K8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L8" t="s">
-        <v>16</v>
-      </c>
-      <c r="M8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="21">
       <c r="A9">
         <f>SUM(A8,10)</f>
         <v>60</v>
@@ -811,27 +818,26 @@
       <c r="F9" s="3">
         <v>5</v>
       </c>
-      <c r="G9" s="3"/>
+      <c r="G9" t="s">
+        <v>16</v>
+      </c>
       <c r="H9" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" t="s">
         <v>17</v>
       </c>
-      <c r="J9">
+      <c r="I9">
         <v>0.2</v>
       </c>
+      <c r="J9" t="s">
+        <v>18</v>
+      </c>
       <c r="K9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L9" t="s">
-        <v>16</v>
-      </c>
-      <c r="M9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="53.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="28" customHeight="1">
       <c r="A10">
         <f t="shared" ref="A10:A11" si="0">SUM(A9,10)</f>
         <v>70</v>
@@ -845,27 +851,26 @@
       <c r="F10" s="3">
         <v>1</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" t="s">
+        <v>16</v>
+      </c>
       <c r="H10" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" t="s">
         <v>17</v>
       </c>
-      <c r="J10">
+      <c r="I10">
         <v>9.6</v>
       </c>
+      <c r="J10" t="s">
+        <v>18</v>
+      </c>
       <c r="K10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="21">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>80</v>
@@ -879,44 +884,30 @@
       <c r="F11" s="3">
         <v>1</v>
       </c>
-      <c r="G11" s="3"/>
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
       <c r="H11" t="s">
-        <v>16</v>
-      </c>
-      <c r="I11" t="s">
         <v>17</v>
       </c>
-      <c r="J11">
+      <c r="I11">
         <v>3.8</v>
       </c>
+      <c r="J11" t="s">
+        <v>18</v>
+      </c>
       <c r="K11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L11" t="s">
-        <v>16</v>
-      </c>
-      <c r="M11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13">
       <c r="E12" s="1"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F10:G10"/>
-  </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>